<commit_message>
Rename provider slug IxDF to IDF across the pipeline
Add map_provider_name() in preprocess.py to rename the raw "IxDF"
provider to "IDF". Update course slugs (IxDF-HCI → IDF-HCI, etc.)
in preprocess.py, constants.py, and aggregate_by_unit.py.

Regenerated all processed data and figures with the corrected names.

https://claude.ai/code/session_01Hv4CTrZoXzk6jvfZNYEZVv
</commit_message>
<xml_diff>
--- a/data/processed/aggregated_by_course_data.xlsx
+++ b/data/processed/aggregated_by_course_data.xlsx
@@ -1517,12 +1517,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>IxDF</t>
+          <t>IDF</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>IxDF-HCI</t>
+          <t>IDF-HCI</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -1825,12 +1825,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>IxDF</t>
+          <t>IDF</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>IxDF-IDU</t>
+          <t>IDF-IDU</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -2133,12 +2133,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>IxDF</t>
+          <t>IDF</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>IxDF-UI</t>
+          <t>IDF-UI</t>
         </is>
       </c>
       <c r="C6" t="n">

</xml_diff>